<commit_message>
scorecard update - first resolved forecasts (LeBron)
</commit_message>
<xml_diff>
--- a/data/final_report.xlsx
+++ b/data/final_report.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,32 +476,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>US-Iran nuclear deal before Jan 20 2029?</t>
+          <t>Exceptional drought — Oregon</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Politics</t>
+          <t>Weather</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>KXUSAIRANAGREEMENT-27-JAN29</t>
+          <t>KXDROUGHTLEVEL-26JULLD4-OR</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>54.0%</t>
+          <t>39.0%</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>22.0%</t>
+          <t>72.0%</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -511,24 +511,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>BUY NO</t>
+          <t>BUY YES</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>1/20/2029</t>
+          <t>7/30/2026</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>-32.0pp</t>
+          <t>+33.0pp</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hormuz traffic normal before Jul 1 2027?</t>
+          <t>Hormuz traffic normal before Jan 1 2027?</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -538,12 +538,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>KXHORMUZNORM-26MAR17-JUL27</t>
+          <t>KXHORMUZNORM-26MAR17-JAN27</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -553,7 +553,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>22.0%</t>
+          <t>30.0%</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -568,19 +568,19 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>7/1/2027</t>
+          <t>1/1/2027</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>-24.0pp</t>
+          <t>-16.0pp</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hormuz traffic normal before Apr 1 2027?</t>
+          <t>U.S. confirms aliens exist before Jan 20 2029?</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -590,22 +590,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>KXHORMUZNORM-26MAR17-APR27</t>
+          <t>KXALIENS-27-JAN29</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>35.0%</t>
+          <t>23.0%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -620,39 +620,39 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>4/1/2027</t>
+          <t>1/20/2029</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>-23.0pp</t>
+          <t>-16.0pp</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Oscar Best Picture — The Odyssey</t>
+          <t>US-Iran nuclear deal before Jan 20 2029?</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Culture</t>
+          <t>Politics</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>KXOSCARPIC-27</t>
+          <t>KXUSAIRANAGREEMENT-27-JAN29</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>55.0%</t>
+          <t>53.0%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -672,44 +672,44 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>3/15/2027</t>
+          <t>1/20/2029</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>-17.0pp</t>
+          <t>-15.0pp</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>U.S. confirms aliens exist before Jan 20 2029?</t>
+          <t>Oscar Best Picture — The Odyssey</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Politics</t>
+          <t>Culture</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>KXALIENS-27-JAN29</t>
+          <t>KXOSCARPIC-27</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>24.0%</t>
+          <t>49.0%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>7.0%</t>
+          <t>37.0%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -724,44 +724,44 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>1/20/2029</t>
+          <t>3/15/2027</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>-17.0pp</t>
+          <t>-12.0pp</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Next Fed rate hike — Before 2027</t>
+          <t>Game Awards 2026 GOTY — Grand Theft Auto VI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Economics</t>
+          <t>Culture</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>KXFEDHIKE-B2027</t>
+          <t>KXGAMEAWARDS-2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>72.0%</t>
+          <t>65.0%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>58.0%</t>
+          <t>53.0%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -776,44 +776,44 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>1/1/2027</t>
+          <t>12/15/2026</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>-14.0pp</t>
+          <t>-12.0pp</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Game Awards 2026 GOTY — Grand Theft Auto VI</t>
+          <t>Next Fed rate hike — Before 2027</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Culture</t>
+          <t>Economics</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>KXGAMEAWARDS-2026</t>
+          <t>KXFEDHIKE-B2027</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>63.0%</t>
+          <t>66.0%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>52.0%</t>
+          <t>54.0%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -828,64 +828,64 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>12/15/2026</t>
+          <t>1/1/2027</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>-11.0pp</t>
+          <t>-12.0pp</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Next James Bond — Callum Turner</t>
+          <t>Fed decision in July — Maintains rate</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Culture</t>
+          <t>Economics</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>KXBOND-30</t>
+          <t>KXFEDDECISION-26JUL-H0</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>38.0%</t>
+          <t>75.0%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>29.0%</t>
+          <t>86.0%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>BUY NO</t>
+          <t>BUY YES</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>1/1/2030</t>
+          <t>7/29/2026</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>-9.0pp</t>
+          <t>+11.0pp</t>
         </is>
       </c>
     </row>
@@ -907,17 +907,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>90.0%</t>
+          <t>91.0%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>81.0%</t>
+          <t>82.0%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -944,32 +944,32 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Fed decision in July — Maintains rate</t>
+          <t>Hormuz traffic normal before Apr 1 2027?</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Economics</t>
+          <t>Politics</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>KXFEDDECISION-26JUL-H0</t>
+          <t>KXHORMUZNORM-26MAR17-APR27</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>53.0%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>84.0%</t>
+          <t>44.0%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -979,17 +979,17 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>BUY YES</t>
+          <t>BUY NO</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>7/29/2026</t>
+          <t>4/1/2027</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>+9.0pp</t>
+          <t>-9.0pp</t>
         </is>
       </c>
     </row>
@@ -1011,12 +1011,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>34.0%</t>
+          <t>35.0%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1041,14 +1041,14 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>-8.0pp</t>
+          <t>-9.0pp</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LeBron James Next Team — Miami Heat</t>
+          <t>F1 Drivers Champion — Andrea Kimi Antonelli</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1058,22 +1058,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>KXNEXTTEAMNBA-26LJAM-MIA</t>
+          <t>KXF1-26-ANT</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>45.0%</t>
+          <t>75.0%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>52.0%</t>
+          <t>70.0%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1083,17 +1083,17 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>BUY YES</t>
+          <t>BUY NO</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>10/1/2026</t>
+          <t>12/7/2026</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>+7.0pp</t>
+          <t>-5.0pp</t>
         </is>
       </c>
     </row>
@@ -1115,17 +1115,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>89.0%</t>
+          <t>85.0%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>84.0%</t>
+          <t>80.0%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1152,27 +1152,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Will the Citrini scenario happen?</t>
+          <t>Big Brother S28 Winner — Dee Valladares</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Economics</t>
+          <t>Culture</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>KXCITRINI-28JUL01</t>
+          <t>KXBIGBROTHER-26DEC31-DV</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>19.0%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1192,49 +1192,49 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>7/1/2028</t>
+          <t>12/31/2026</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>-5.0pp</t>
+          <t>-4.0pp</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CA 8.0+ earthquake before 2027?</t>
+          <t>2027 NBA Champion — San Antonio Spurs</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Weather</t>
+          <t>Sports</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>KXEARTHQUAKECALIFORNIA-27</t>
+          <t>KXNBA-27-SAS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>7.0%</t>
+          <t>21.0%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2.0%</t>
+          <t>17.0%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1244,44 +1244,44 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>1/1/2027</t>
+          <t>6/30/2027</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>-5.0pp</t>
+          <t>-4.0pp</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Exceptional drought — Oregon</t>
+          <t>Number of rate cuts in 2026 — Exactly 0</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Weather</t>
+          <t>Economics</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>KXDROUGHTLEVEL-26JULLD4-OR</t>
+          <t>KXRATECUTCOUNT-26DEC31</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>29.0%</t>
+          <t>80.0%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>24.0%</t>
+          <t>84.0%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1291,49 +1291,49 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>BUY NO</t>
+          <t>BUY YES</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>7/30/2026</t>
+          <t>12/31/2026</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>-5.0pp</t>
+          <t>+4.0pp</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Number of rate cuts in 2026 — Exactly 0</t>
+          <t>CA 8.0+ earthquake before 2027?</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Economics</t>
+          <t>Weather</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>KXRATECUTCOUNT-26DEC31</t>
+          <t>KXEARTHQUAKECALIFORNIA-27</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>83.0%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>87.0%</t>
+          <t>2.0%</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1343,49 +1343,49 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>BUY YES</t>
+          <t>BUY NO</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>12/31/2026</t>
+          <t>1/1/2027</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>+4.0pp</t>
+          <t>-3.0pp</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2027 NFL Champion — LA Rams</t>
+          <t>Will the Citrini scenario happen?</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Sports</t>
+          <t>Economics</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>KXSB-27-LAR</t>
+          <t>KXCITRINI-28JUL01</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>17.0%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>14.0%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2/14/2027</t>
+          <t>7/1/2028</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1412,7 +1412,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2027 Pro Basketball Champion — OKC Thunder</t>
+          <t>2027 NFL Champion — LA Rams</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1422,22 +1422,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>KXNBA-27-OKC</t>
+          <t>KXSB-27-LAR</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>21.0%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1452,7 +1452,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>6/30/2027</t>
+          <t>2/14/2027</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1516,32 +1516,32 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Stranger Things new episode this year?</t>
+          <t>Rain in Seattle this month — Above 1 inch</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Culture</t>
+          <t>Weather</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>KXMEDIARELEASEST-27JAN01</t>
+          <t>KXRAINSEAM-26JUL-1</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>2.0%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1/1/2027</t>
+          <t>7/31/2026</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1568,32 +1568,32 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>More tech layoffs in 2026 than in 2025?</t>
+          <t>Stranger Things new episode this year?</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Economics</t>
+          <t>Culture</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>KXLAYOFFSYINFO-26</t>
+          <t>KXMEDIARELEASEST-27JAN01</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>89.0%</t>
+          <t>6.0%</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>89.0%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1608,44 +1608,44 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>3/1/2027</t>
+          <t>1/1/2027</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>+0.0pp</t>
+          <t>-1.0pp</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Hurricane Bertha — Category 1 or above</t>
+          <t>College Football Champion — Ohio State</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Weather</t>
+          <t>Sports</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>KXHURCAT-26BERTHA</t>
+          <t>KXNCAAF-27-OSU</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>7/24/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.0%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>1.0%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1660,62 +1660,114 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>12/1/2026</t>
+          <t>1/15/2027</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>+0.0pp</t>
+          <t>-1.0pp</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>More tech layoffs in 2026 than in 2025?</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Economics</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>KXLAYOFFSYINFO-26</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>7/27/2026</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>89.0%</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>89.0%</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>SPECULATIVE</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>NO TRADE</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>3/1/2027</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>+0.0pp</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>First Atlantic hurricane — Cristobal</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>Weather</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>KXFIRSTHURRICANE-26DEC01ATL</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>7/24/2026</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>53.0%</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>53.0%</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>7/27/2026</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>47.0%</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>47.0%</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
         <is>
           <t>SPECULATIVE</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>NO TRADE</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>12/1/2026</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>+0.0pp</t>
         </is>

</xml_diff>

<commit_message>
Aug 10 cycle - Blanche resolved correct
</commit_message>
<xml_diff>
--- a/data/final_report.xlsx
+++ b/data/final_report.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,7 +476,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Hormuz traffic normal before Dec 1 2026?</t>
+          <t>U.S. confirms aliens exist before Jan 20 2029?</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -486,22 +486,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>KXHORMUZNORM-26MAR17-DEC26</t>
+          <t>KXALIENS-27-JAN29</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>42.0%</t>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>27.0%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -516,19 +516,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2029-01-20</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>-15.0pp</t>
+          <t>-18.0pp</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hormuz traffic normal before Jan 1 2027?</t>
+          <t>Hormuz traffic normal before Apr 1 2027?</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -538,22 +538,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>KXHORMUZNORM-26MAR17-JAN27</t>
+          <t>KXHORMUZNORM-26MAR17-APR27</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>49.0%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>34.0%</t>
+          <t>36.0%</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -568,19 +568,19 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-04-01</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>-15.0pp</t>
+          <t>-14.0pp</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Game Awards 2026 GOTY — Grand Theft Auto VI</t>
+          <t>Oscar Best Picture — The Odyssey</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -590,22 +590,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>KXGAMEAWARDS-2026</t>
+          <t>KXOSCARPIC-27</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>68.0%</t>
+          <t>49.0%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>54.0%</t>
+          <t>36.0%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -620,44 +620,44 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-12-15</t>
+          <t>2027-03-15</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>-14.0pp</t>
+          <t>-13.0pp</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>U.S. confirms aliens exist before Jan 20 2029?</t>
+          <t>Fed decision in September — Maintains rate</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Politics</t>
+          <t>Economics</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>KXALIENS-27-JAN29</t>
+          <t>KXFEDDECISION-26SEP-H0</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>21.0%</t>
+          <t>65.0%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>7.0%</t>
+          <t>77.0%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -667,49 +667,49 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>BUY NO</t>
+          <t>BUY YES</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2029-01-20</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>-14.0pp</t>
+          <t>+12.0pp</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Fed decision in September — Maintains rate</t>
+          <t>Pro Baseball Champion — Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Economics</t>
+          <t>Sports</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>KXFEDDECISION-26SEP-H0</t>
+          <t>KXMLB-26-LAD</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>64.0%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>76.0%</t>
+          <t>28.0%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -719,49 +719,49 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>BUY YES</t>
+          <t>BUY NO</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>+12.0pp</t>
+          <t>-12.0pp</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Oscar Best Picture — The Odyssey</t>
+          <t>US-Iran nuclear deal before Jan 20 2029?</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Culture</t>
+          <t>Politics</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>KXOSCARPIC-27</t>
+          <t>KXUSAIRANAGREEMENT-27-JAN29</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>48.0%</t>
+          <t>51.0%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>36.0%</t>
+          <t>39.0%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2027-03-15</t>
+          <t>2029-01-20</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -788,37 +788,37 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>US-Iran nuclear deal before Jan 20 2029?</t>
+          <t>Will 2026 be the hottest year ever?</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Politics</t>
+          <t>Weather</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>KXUSAIRANAGREEMENT-27-JAN29</t>
+          <t>KXGTEMP-26</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>51.0%</t>
+          <t>68.0%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>39.0%</t>
+          <t>58.0%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -828,49 +828,49 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2029-01-20</t>
+          <t>2027-01-15</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>-12.0pp</t>
+          <t>-10.0pp</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Will 2026 be the hottest year ever?</t>
+          <t>Hormuz traffic normal before Jul 1 2027?</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Weather</t>
+          <t>Politics</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>KXGTEMP-26</t>
+          <t>KXHORMUZNORM-26MAR17-JUL27</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>69.0%</t>
+          <t>56.0%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>58.0%</t>
+          <t>46.0%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -880,12 +880,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2027-01-15</t>
+          <t>2027-07-01</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>-11.0pp</t>
+          <t>-10.0pp</t>
         </is>
       </c>
     </row>
@@ -907,17 +907,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>90.0%</t>
+          <t>88.0%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>79.0%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -937,44 +937,44 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>-10.0pp</t>
+          <t>-9.0pp</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Pro Baseball Champion — Los Angeles Dodgers</t>
+          <t>Leaders leaving office 2026 — Benjamin Netanyahu</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Sports</t>
+          <t>Politics</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>KXMLB-26-LAD</t>
+          <t>KXLEADERSOUT-26-BN</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>37.0%</t>
+          <t>46.0%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>27.0%</t>
+          <t>38.0%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -984,96 +984,96 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>-10.0pp</t>
+          <t>-8.0pp</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Will the Citrini scenario happen?</t>
+          <t>This July 2026 is the hottest July ever?</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Economics</t>
+          <t>Weather</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>KXCITRINI-28JUL01</t>
+          <t>KXHIGHJULY-26</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>21.0%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>14.0%</t>
+          <t>24.0%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>BUY NO</t>
+          <t>BUY YES</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2028-07-01</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>-7.0pp</t>
+          <t>+8.0pp</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Trump next Attorney General — Todd Blanche</t>
+          <t>Next James Bond — Callum Turner</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Politics</t>
+          <t>Culture</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>KXNEXTAG-29-TB</t>
+          <t>KXBOND-30-CT</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>81.0%</t>
+          <t>36.0%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>88.0%</t>
+          <t>28.0%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1083,24 +1083,24 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>BUY YES</t>
+          <t>BUY NO</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2029-01-20</t>
+          <t>2030-01-01</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>+7.0pp</t>
+          <t>-8.0pp</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Next Fed rate hike — Before 2027</t>
+          <t>Will the Citrini scenario happen?</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1110,27 +1110,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>KXFEDHIKE-B2027</t>
+          <t>KXCITRINI-28JUL01</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>55.0%</t>
+          <t>19.0%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1140,12 +1140,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2028-07-01</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>-5.0pp</t>
+          <t>-6.0pp</t>
         </is>
       </c>
     </row>
@@ -1167,12 +1167,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>24.0%</t>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1197,39 +1197,39 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>-5.0pp</t>
+          <t>-6.0pp</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Big Brother S28 Winner — Dee Valladares</t>
+          <t>Next Fed rate hike — Before 2027</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Culture</t>
+          <t>Economics</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>KXBIGBROTHER-26DEC31-DV</t>
+          <t>KXFEDHIKE-B2027</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>23.0%</t>
+          <t>55.0%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>19.0%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1244,44 +1244,44 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-12-31</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>-4.0pp</t>
+          <t>-5.0pp</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CA 8.0+ earthquake before 2027?</t>
+          <t>Big Brother S28 Winner — Dee Valladares</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Weather</t>
+          <t>Culture</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>KXEARTHQUAKECALIFORNIA-27</t>
+          <t>KXBIGBROTHER-26DEC31-DV</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>23.0%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2.0%</t>
+          <t>19.0%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1296,7 +1296,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1360,7 +1360,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2027 NFL Champion — LA Rams</t>
+          <t>F1 Drivers Champion — Andrea Kimi Antonelli</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1370,22 +1370,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>KXSB-27-LAR</t>
+          <t>KXF1-26-ANT</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>74.0%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>71.0%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2027-02-14</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1412,188 +1412,188 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>College Football Champion — Notre Dame</t>
+          <t>CA 8.0+ earthquake before 2027?</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Sports</t>
+          <t>Weather</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>KXNCAAF-27-ND</t>
+          <t>KXEARTHQUAKECALIFORNIA-27</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>2.0%</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>SPECULATIVE</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>NO TRADE</t>
+          <t>BUY NO</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2027-01-15</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>-2.0pp</t>
+          <t>-3.0pp</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>More tech layoffs in 2026 than in 2025?</t>
+          <t>2027 NFL Champion — LA Rams</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Economics</t>
+          <t>Sports</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>KXLAYOFFSYINFO-26</t>
+          <t>KXSB-27-LAR</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>91.0%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>90.0%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>SPECULATIVE</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>NO TRADE</t>
+          <t>BUY NO</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2027-03-01</t>
+          <t>2027-02-14</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-1.0pp</t>
+          <t>-3.0pp</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Will the SAVE Act become law?</t>
+          <t>College Football Champion — Notre Dame</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Politics</t>
+          <t>Sports</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>KXSAVEACT-27</t>
+          <t>KXNCAAF-27-ND</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>SPECULATIVE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>BUY NO</t>
+          <t>NO TRADE</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2027-01-04</t>
+          <t>2027-01-15</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-1.0pp</t>
+          <t>-2.0pp</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Stranger Things new episode this year?</t>
+          <t>More tech layoffs in 2026 than in 2025?</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Culture</t>
+          <t>Economics</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>KXMEDIARELEASEST-27JAN01</t>
+          <t>KXLAYOFFSYINFO-26</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>92.0%</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>91.0%</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1608,114 +1608,166 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-03-01</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>+0.0pp</t>
+          <t>-1.0pp</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>First Atlantic hurricane — Cristobal</t>
+          <t>Will the SAVE Act become law?</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Weather</t>
+          <t>Politics</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>KXFIRSTHURRICANE-26DEC01ATL</t>
+          <t>KXSAVEACT-27</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>45.0%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>45.0%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>SPECULATIVE</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>NO TRADE</t>
+          <t>BUY NO</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2027-01-04</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>+0.0pp</t>
+          <t>-1.0pp</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Highest temp in LA today — 79-80</t>
+          <t>Stranger Things new episode this year?</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>Culture</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>KXMEDIARELEASEST-27JAN01</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>4.0%</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>4.0%</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>SPECULATIVE</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>NO TRADE</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>+0.0pp</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>First Atlantic hurricane — Cristobal</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
           <t>Weather</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>KXHIGHLAX-26AUG07</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>52.0%</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>52.0%</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>KXFIRSTHURRICANE-26DEC01ATL</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>38.0%</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>38.0%</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
         <is>
           <t>SPECULATIVE</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>NO TRADE</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
         <is>
           <t>+0.0pp</t>
         </is>

</xml_diff>

<commit_message>
fix STOP guard allowlist, revert Spider-Man
</commit_message>
<xml_diff>
--- a/data/final_report.xlsx
+++ b/data/final_report.xlsx
@@ -476,32 +476,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>U.S. confirms aliens exist before Jan 20 2029?</t>
+          <t>Oscar Best Picture — The Odyssey</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Politics</t>
+          <t>Culture</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>KXALIENS-27-JAN29</t>
+          <t>KXOSCARPIC-27</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>54.0%</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>7.0%</t>
+          <t>37.0%</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -516,19 +516,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2029-01-20</t>
+          <t>2027-03-15</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>-18.0pp</t>
+          <t>-17.0pp</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hormuz traffic normal before Apr 1 2027?</t>
+          <t>U.S. confirms aliens exist before Jan 20 2029?</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -538,22 +538,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>KXHORMUZNORM-26MAR17-APR27</t>
+          <t>KXALIENS-27-JAN29</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>23.0%</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>36.0%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -568,44 +568,44 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2027-04-01</t>
+          <t>2029-01-20</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>-14.0pp</t>
+          <t>-16.0pp</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Oscar Best Picture — The Odyssey</t>
+          <t>Hormuz traffic normal before Apr 1 2027?</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Culture</t>
+          <t>Politics</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>KXOSCARPIC-27</t>
+          <t>KXHORMUZNORM-26MAR17-APR27</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>49.0%</t>
+          <t>48.0%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>36.0%</t>
+          <t>35.0%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -620,7 +620,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2027-03-15</t>
+          <t>2027-04-01</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -632,32 +632,32 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Fed decision in September — Maintains rate</t>
+          <t>US-Iran nuclear deal before Jan 20 2029?</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Economics</t>
+          <t>Politics</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>KXFEDDECISION-26SEP-H0</t>
+          <t>KXUSAIRANAGREEMENT-27-JAN29</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>65.0%</t>
+          <t>51.0%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>77.0%</t>
+          <t>39.0%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -667,49 +667,49 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>BUY YES</t>
+          <t>BUY NO</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2029-01-20</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>+12.0pp</t>
+          <t>-12.0pp</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pro Baseball Champion — Los Angeles Dodgers</t>
+          <t>Fed decision in September — Maintains rate</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sports</t>
+          <t>Economics</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>KXMLB-26-LAD</t>
+          <t>KXFEDDECISION-26SEP-H0</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>65.0%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>28.0%</t>
+          <t>77.0%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -719,49 +719,49 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>BUY NO</t>
+          <t>BUY YES</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>-12.0pp</t>
+          <t>+12.0pp</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>US-Iran nuclear deal before Jan 20 2029?</t>
+          <t>Next James Bond — Jack Lowden</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Politics</t>
+          <t>Culture</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>KXUSAIRANAGREEMENT-27-JAN29</t>
+          <t>KXBOND-30-JL</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>51.0%</t>
+          <t>37.0%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>39.0%</t>
+          <t>26.0%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -776,49 +776,49 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2029-01-20</t>
+          <t>2030-01-01</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>-12.0pp</t>
+          <t>-11.0pp</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Will 2026 be the hottest year ever?</t>
+          <t>Pro Baseball Champion — Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Weather</t>
+          <t>Sports</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>KXGTEMP-26</t>
+          <t>KXMLB-26-LAD</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>68.0%</t>
+          <t>37.0%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>58.0%</t>
+          <t>27.0%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -828,7 +828,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2027-01-15</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -855,17 +855,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>56.0%</t>
+          <t>53.0%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>46.0%</t>
+          <t>44.0%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -885,44 +885,44 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>-10.0pp</t>
+          <t>-9.0pp</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GTA VI release before 2027?</t>
+          <t>Will 2026 be the hottest year ever?</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Culture</t>
+          <t>Weather</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>KXGTA6-B2027</t>
+          <t>KXGTEMP-26</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>88.0%</t>
+          <t>65.0%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>79.0%</t>
+          <t>57.0%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -932,19 +932,19 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-01-15</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>-9.0pp</t>
+          <t>-8.0pp</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Leaders leaving office 2026 — Benjamin Netanyahu</t>
+          <t>Leaders leaving office 2026 — Christopher Luxon</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -954,22 +954,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>KXLEADERSOUT-26-BN</t>
+          <t>KXLEADERSOUT-27JAN01-CL</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>46.0%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>38.0%</t>
+          <t>42.0%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -996,89 +996,89 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>This July 2026 is the hottest July ever?</t>
+          <t>GTA VI release before 2027?</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Weather</t>
+          <t>Culture</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>KXHIGHJULY-26</t>
+          <t>KXGTA6-B2027</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>87.0%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>24.0%</t>
+          <t>79.0%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>BUY YES</t>
+          <t>BUY NO</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>+8.0pp</t>
+          <t>-8.0pp</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Next James Bond — Callum Turner</t>
+          <t>Will the Citrini scenario happen?</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Culture</t>
+          <t>Economics</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>KXBOND-30-CT</t>
+          <t>KXCITRINI-28JUL01</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>36.0%</t>
+          <t>20.0%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>28.0%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1088,49 +1088,49 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2030-01-01</t>
+          <t>2028-07-01</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>-8.0pp</t>
+          <t>-7.0pp</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Will the Citrini scenario happen?</t>
+          <t>Big Brother S28 Winner — Dee Valladares</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Economics</t>
+          <t>Culture</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>KXCITRINI-28JUL01</t>
+          <t>KXBIGBROTHER-26DEC31-DV</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>19.0%</t>
+          <t>27.0%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>21.0%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2028-07-01</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1167,12 +1167,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>24.0%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1197,39 +1197,39 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>-6.0pp</t>
+          <t>-5.0pp</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Next Fed rate hike — Before 2027</t>
+          <t>CA 8.0+ earthquake before 2027?</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Economics</t>
+          <t>Weather</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>KXFEDHIKE-B2027</t>
+          <t>KXEARTHQUAKECALIFORNIA-27</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>55.0%</t>
+          <t>6.0%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>2.0%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1249,39 +1249,39 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>-5.0pp</t>
+          <t>-4.0pp</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Big Brother S28 Winner — Dee Valladares</t>
+          <t>Number of rate cuts in 2026 — Exactly 0</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Culture</t>
+          <t>Economics</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>KXBIGBROTHER-26DEC31-DV</t>
+          <t>KXRATECUTCOUNT-26DEC31</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>23.0%</t>
+          <t>86.0%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>19.0%</t>
+          <t>89.0%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>BUY NO</t>
+          <t>BUY YES</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1301,39 +1301,39 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>-4.0pp</t>
+          <t>+3.0pp</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Number of rate cuts in 2026 — Exactly 0</t>
+          <t>2027 NFL Champion — LA Rams</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Economics</t>
+          <t>Sports</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>KXRATECUTCOUNT-26DEC31</t>
+          <t>KXSB-27-LAR</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>86.0%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>89.0%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1343,24 +1343,24 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>BUY YES</t>
+          <t>BUY NO</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-12-31</t>
+          <t>2027-02-14</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>+3.0pp</t>
+          <t>-3.0pp</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>F1 Drivers Champion — Andrea Kimi Antonelli</t>
+          <t>FedEx St. Jude Championship — Scottie Scheffler</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1370,22 +1370,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>KXF1-26-ANT</t>
+          <t>KXPGATOUR-FESJC26-SS</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>74.0%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>71.0%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-12-07</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1412,7 +1412,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CA 8.0+ earthquake before 2027?</t>
+          <t>This July 2026 is the hottest July ever?</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1422,94 +1422,94 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>KXEARTHQUAKECALIFORNIA-27</t>
+          <t>KXHMONTH-26JUL</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>23.0%</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2.0%</t>
+          <t>26.0%</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>SPECULATIVE</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>BUY NO</t>
+          <t>NO TRADE</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>-3.0pp</t>
+          <t>+3.0pp</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2027 NFL Champion — LA Rams</t>
+          <t>Next Fed rate hike — Before 2027</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Sports</t>
+          <t>Economics</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>KXSB-27-LAR</t>
+          <t>KXFEDHIKE-B2027</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>52.0%</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>SPECULATIVE</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>BUY NO</t>
+          <t>NO TRADE</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2027-02-14</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-3.0pp</t>
+          <t>-2.0pp</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1568,32 +1568,32 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>More tech layoffs in 2026 than in 2025?</t>
+          <t>Will the SAVE Act become law?</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Economics</t>
+          <t>Politics</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>KXLAYOFFSYINFO-26</t>
+          <t>KXSAVEACT-27</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>92.0%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>91.0%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2027-03-01</t>
+          <t>2027-01-04</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1620,52 +1620,52 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Will the SAVE Act become law?</t>
+          <t>More tech layoffs in 2026 than in 2025?</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Politics</t>
+          <t>Economics</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>KXSAVEACT-27</t>
+          <t>KXLAYOFFSYINFO-26</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>91.0%</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>91.0%</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>SPECULATIVE</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>BUY NO</t>
+          <t>NO TRADE</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2027-01-04</t>
+          <t>2027-03-01</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>-1.0pp</t>
+          <t>+0.0pp</t>
         </is>
       </c>
     </row>
@@ -1687,17 +1687,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1739,17 +1739,17 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>38.0%</t>
+          <t>33.0%</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>38.0%</t>
+          <t>33.0%</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">

</xml_diff>